<commit_message>
Gas reading 11639.674 m3 on 2026-10-15 08:10, projections refreshed
Dictated by Marton; appended via add-meter skill, iter1-5 rerun.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/gaz.xlsx
+++ b/inst/extdata/gaz.xlsx
@@ -6024,6 +6024,74 @@
         <v>0.562406886747753</v>
       </c>
     </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>11619.71</v>
+      </c>
+      <c r="B334" s="1" t="n">
+        <v>46288.2777777778</v>
+      </c>
+      <c r="C334" t="n">
+        <v>25.6099999999988</v>
+      </c>
+      <c r="D334" t="n">
+        <v>37.5701388888889</v>
+      </c>
+      <c r="E334" t="n">
+        <v>0.6816583796972</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>11626.17</v>
+      </c>
+      <c r="B335" s="1" t="n">
+        <v>46298.2416666667</v>
+      </c>
+      <c r="C335" t="n">
+        <v>6.46000000000095</v>
+      </c>
+      <c r="D335" t="n">
+        <v>9.96388888888889</v>
+      </c>
+      <c r="E335" t="n">
+        <v>0.648341232227583</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>11634.83</v>
+      </c>
+      <c r="B336" s="1" t="n">
+        <v>46306.6930555556</v>
+      </c>
+      <c r="C336" t="n">
+        <v>8.65999999999985</v>
+      </c>
+      <c r="D336" t="n">
+        <v>8.45138888888889</v>
+      </c>
+      <c r="E336" t="n">
+        <v>1.02468364831551</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>11639.674</v>
+      </c>
+      <c r="B337" s="1" t="n">
+        <v>46310.2569444444</v>
+      </c>
+      <c r="C337" t="n">
+        <v>4.84400000000096</v>
+      </c>
+      <c r="D337" t="n">
+        <v>3.56388888888889</v>
+      </c>
+      <c r="E337" t="n">
+        <v>1.35918939984438</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Gas reading 11667.0045 m3 on 2026-10-25 09:03, projections refreshed
Dictated by Marton; appended via add-meter, iter1-5 rerun (DIAL DOWN, ~44%
chance of exceeding the 1,729 m3 quota). His other pending edits left as they are.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/gaz.xlsx
+++ b/inst/extdata/gaz.xlsx
@@ -6092,6 +6092,23 @@
         <v>1.35918939984438</v>
       </c>
     </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>11667.0045</v>
+      </c>
+      <c r="B338" s="1" t="n">
+        <v>46320.3354166667</v>
+      </c>
+      <c r="C338" t="n">
+        <v>27.3304999999982</v>
+      </c>
+      <c r="D338" t="n">
+        <v>10.0784722222222</v>
+      </c>
+      <c r="E338" t="n">
+        <v>2.71177013711827</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>